<commit_message>
ran s6 and tracked more files to review
</commit_message>
<xml_diff>
--- a/outputs/tables/table1_employment_exports.xlsx
+++ b/outputs/tables/table1_employment_exports.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Table1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,17 +419,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>country</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Total_employment_THS</t>
+          <t>total_employment_THS</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Exports_to_nonEU_MIO_EUR</t>
+          <t>exports_to_nonEU_MIO_EUR</t>
         </is>
       </c>
     </row>
@@ -443,7 +443,7 @@
         <v>4031.83</v>
       </c>
       <c r="C2" t="n">
-        <v>42281.61</v>
+        <v>42281.614</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>4473.8</v>
       </c>
       <c r="C3" t="n">
-        <v>76051.25</v>
+        <v>76051.24799999999</v>
       </c>
     </row>
     <row r="4">
@@ -469,7 +469,7 @@
         <v>3574.94</v>
       </c>
       <c r="C4" t="n">
-        <v>7595.27</v>
+        <v>7595.271000000001</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v>404.3</v>
       </c>
       <c r="C5" t="n">
-        <v>4221.73</v>
+        <v>4221.732</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         <v>4954.56</v>
       </c>
       <c r="C6" t="n">
-        <v>21291.17</v>
+        <v>21291.174</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         <v>40636</v>
       </c>
       <c r="C7" t="n">
-        <v>408951.28</v>
+        <v>408951.281</v>
       </c>
     </row>
     <row r="8">
@@ -521,7 +521,7 @@
         <v>2746.02</v>
       </c>
       <c r="C8" t="n">
-        <v>52771.93</v>
+        <v>52771.931</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>559.7</v>
       </c>
       <c r="C9" t="n">
-        <v>3865.71</v>
+        <v>3865.714</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>4694</v>
       </c>
       <c r="C10" t="n">
-        <v>23657.8</v>
+        <v>23657.804</v>
       </c>
     </row>
     <row r="11">
@@ -560,7 +560,7 @@
         <v>19423.8</v>
       </c>
       <c r="C11" t="n">
-        <v>104715.19</v>
+        <v>104715.189</v>
       </c>
     </row>
     <row r="12">
@@ -573,7 +573,7 @@
         <v>2466.6</v>
       </c>
       <c r="C12" t="n">
-        <v>36290.28</v>
+        <v>36290.279</v>
       </c>
     </row>
     <row r="13">
@@ -586,7 +586,7 @@
         <v>26599.2</v>
       </c>
       <c r="C13" t="n">
-        <v>240850.64</v>
+        <v>240850.639</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>1666.38</v>
       </c>
       <c r="C14" t="n">
-        <v>3871.79</v>
+        <v>3871.791</v>
       </c>
     </row>
     <row r="15">
@@ -612,7 +612,7 @@
         <v>3858.5</v>
       </c>
       <c r="C15" t="n">
-        <v>21977.86</v>
+        <v>21977.864</v>
       </c>
     </row>
     <row r="16">
@@ -625,7 +625,7 @@
         <v>1913.5</v>
       </c>
       <c r="C16" t="n">
-        <v>86153.34</v>
+        <v>86153.345</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         <v>24413.4</v>
       </c>
       <c r="C17" t="n">
-        <v>186940.65</v>
+        <v>186940.651</v>
       </c>
     </row>
     <row r="18">
@@ -651,7 +651,7 @@
         <v>1234.44</v>
       </c>
       <c r="C18" t="n">
-        <v>6571.74</v>
+        <v>6571.737999999999</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         <v>255.79</v>
       </c>
       <c r="C19" t="n">
-        <v>20587.88</v>
+        <v>20587.876</v>
       </c>
     </row>
     <row r="20">
@@ -677,7 +677,7 @@
         <v>824.55</v>
       </c>
       <c r="C20" t="n">
-        <v>3344.93</v>
+        <v>3344.927</v>
       </c>
     </row>
     <row r="21">
@@ -690,7 +690,7 @@
         <v>135.09</v>
       </c>
       <c r="C21" t="n">
-        <v>2341.64</v>
+        <v>2341.639</v>
       </c>
     </row>
     <row r="22">
@@ -703,7 +703,7 @@
         <v>8702</v>
       </c>
       <c r="C22" t="n">
-        <v>101955.4</v>
+        <v>101955.397</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         <v>15202.8</v>
       </c>
       <c r="C23" t="n">
-        <v>41791.16</v>
+        <v>41791.157</v>
       </c>
     </row>
     <row r="24">
@@ -726,10 +726,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4843.13</v>
+        <v>4843.130000000001</v>
       </c>
       <c r="C24" t="n">
-        <v>15917.36</v>
+        <v>15917.356</v>
       </c>
     </row>
     <row r="25">
@@ -742,7 +742,7 @@
         <v>8698.1</v>
       </c>
       <c r="C25" t="n">
-        <v>13596.44</v>
+        <v>13596.444</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         <v>4226</v>
       </c>
       <c r="C26" t="n">
-        <v>74466.14999999999</v>
+        <v>74466.152</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         <v>957.89</v>
       </c>
       <c r="C27" t="n">
-        <v>6167.62</v>
+        <v>6167.625</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>2147.89</v>
       </c>
       <c r="C28" t="n">
-        <v>9544.379999999999</v>
+        <v>9544.377</v>
       </c>
     </row>
     <row r="29">
@@ -794,7 +794,7 @@
         <v>24562.93</v>
       </c>
       <c r="C29" t="n">
-        <v>253478.52</v>
+        <v>253478.519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>